<commit_message>
Standards research in lockstep with the app (plan 61, 2026-10-03)
- Operator (scripts/apply-standards-research-2026-10-03.py, expect-then-set
  guards): Pararescue on the 2023 IFT (run 10:20, swim 12:30, push-ups 40,
  sit-ups 50, pull-ups "(2 min)"), broad jump (general 1.70/1.95/2.20/2.40,
  special forces 1.93/2.16/2.39/2.65), police plank 1:30/2:30/3:30/4:30, USMC
  plank Pass 1:10; the app's cites copied into a new cite column.
- Lift: HYROX Open lower tiers (men and women), Cindy's note, the site's own
  broad jump men's Elite 2.85 -> 2.75, and three base cells the app moved
  (women's OHP Beginner 25 kg, women's 20 / 40 km TT Beginner).
- New check:app-lift (WODs, base table, pathway overrides vs the app);
  check:app-ors also compares cites. Both: 0 differences.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,6 +551,18 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Cream-filled cell = value to be populated (TODO). Red text = legal/commercial caution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Change 2026-10-03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mirrors the TPF app's plan 61 (tpf-app docs/build/61_MISSING_STANDARDS_RESEARCH_2026-10-03.md section 8). HYROX race: men Beginner 1:57:30 and Novice 1:37:30 (3.9 x TPF's 5 km), women Beginner 2:09:30, Novice 1:47:30, Experienced 1:34:30 (men x 1.10); every tier now has a permitted basis. Cindy kept, now checked. TPF Benchmark's own broad jump: men's Elite 285 -&gt; 275 cm, relabelled TPF's own, now checked. The HABS base table follows the app: women's overhead press Beginner 20 -&gt; 25 kg, women's 20 km TT Beginner 50:00 -&gt; 49:30 (40 km derived: 1:42:30). Script: scripts/apply-standards-research-2026-10-03.py.</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1160,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>TPF's own ladder. No openly licensed population norm exists; checked only against published ratios (women's overhead press ≈ 0.5-0.6 of men's absolute — Nuzzo 2023 review) and the CrossFit sample of Meier, Rabel, Schmidt 2021 (Sports 9:80, CC BY)</t>
+          <t>TPF's own ladder. No openly licensed population norm exists. Checked 2026-10-03 (tpf-app plan 61 Part C §2.2) against TPF's own bench / squat / deadlift ladders x the overhead-press ratios of the CrossFit samples of Meier, Rabel, Schmidt 2021 (Sports 9:80) and Dexheimer 2019 (both CC BY): the men's ladder reproduced to within 2.5 kg; the women's Beginner 20 -&gt; 25 kg (the empty bar sat below every anchor, 23-30 kg). Women's ≈ 0.5-0.6 of men's absolute (Nuzzo 2023 review)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1168,7 +1180,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Owner-set; ratio checks only (2026-10-02)</t>
+          <t>Owner-set; ratio checks (2026-10-03)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1448,7 +1460,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set). No openly licensed population table has been checked yet (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 (tpf-app plan 61 Part B §3.3) against Norwegian conscripts 2020 (Aandstad et al. 2023, Scand J Med Sci Sports, CC BY 4.0), US Army Ranger course candidates (Physiol Rep 2026, CC BY), Serbian police students (through a CC BY review, Healthcare 2023), AFSPECWAR candidates (Feeney et al. 2023, facts) and China's National Student Physical Health Standard (2014 revision, a Ministry of Education standard). Men's Elite 285 -&gt; 275 cm (2.85 m sat above every anchor); the women's ladder kept, about 0.80 x the men's at every tier</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1468,7 +1480,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Expert-set (TPF)</t>
+          <t>Expert-set (TPF); checked against permitted anchors (2026-10-03)</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2103,7 +2115,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>TPF's own triathlete-pathway anchor (round 13: elite 27:00 M ≈ 44 km/h). No permitted anchor yet (a gap)</t>
+          <t>TPF's own triathlete-pathway anchor (round 13: elite 27:00 M ≈ 44 km/h), checked 2026-10-03 (tpf-app plan 61 Part C §4): Beginner at the US Army AFT 12 km stationary-bike pass time (2025 tables, a US government work) scaled to 20 km (Riegel exp 1.05) — men 45:10, women 49:32, so the women's Beginner moved 50:00 -&gt; 49:30; Elite graded against the UCI Hour Records (facts) — men's Elite 74 % of world best; sex gap 1.11. Assumes a time-trial bike (or clip-on aero bars), a flat course and still air</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2123,7 +2135,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Owner-set (TPF)</t>
+          <t>Owner-set (TPF); checked against permitted anchors (2026-10-03)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3190,7 +3202,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>TPF's own; no openly licensed norm — ratio checks only (2026-10-02)</t>
+          <t>TPF's own; no openly licensed norm — checked 2026-10-03 against the CrossFit overhead-press ratios (Meier 2021, Dexheimer 2019, CC BY): reproduced to within 2.5 kg, kept (tpf-app plan 61 Part C §2.2)</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3226,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F20" t="n">
         <v>30</v>
@@ -3236,7 +3248,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>TPF's own; no openly licensed norm — ratio checks only (2026-10-02)</t>
+          <t>TPF's own; no openly licensed norm — checked 2026-10-03 against the CrossFit overhead-press ratios (Meier 2021, Dexheimer 2019, CC BY): Beginner 20 -&gt; 25 kg, the empty bar sat below every anchor (tpf-app plan 61 Part C §2.2). The HYROX, triathlete and bodybuilder pathways keep their own 20 kg (an owner question in the app's record)</t>
         </is>
       </c>
     </row>
@@ -3646,16 +3658,16 @@
         <v>270</v>
       </c>
       <c r="K29" t="n">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no permitted table checked yet (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 against permitted anchors (Norwegian conscripts, Aandstad 2023, CC BY; US Army Ranger candidates, 2026, CC BY; China's student standard, 2014) — tpf-app plan 61 Part B §3.3</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>novice/intermediate/advanced interpolated from pass/good/excellent/elite (2026-08-07)</t>
+          <t>novice/intermediate/advanced interpolated from pass/good/excellent/elite (2026-08-07); Elite 285 -&gt; 275 cm 2026-10-03 (tpf-app plan 61 Part B §3.3: 2.85 m sat above every anchor; the women's 220 keeps a 0.80 ratio)</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3713,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no permitted table checked yet (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 against permitted anchors (Norwegian conscripts, Aandstad 2023, CC BY; US Army Ranger candidates, 2026, CC BY; China's student standard, 2014) — tpf-app plan 61 Part B §3.3</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4666,7 +4678,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>TPF's own (round 13); no permitted anchor yet (a gap)</t>
+          <t>TPF's own (round 13); checked 2026-10-03: Beginner at the US Army AFT 12 km bike pass scaled to 20 km (45:10), Elite graded against the UCI Hour Records; a TT bike, flat, still air (tpf-app plan 61 Part C §4)</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -4696,7 +4708,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>50:00</t>
+          <t>49:30</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4731,7 +4743,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>TPF's own (round 13); no permitted anchor yet (a gap)</t>
+          <t>TPF's own (round 13); checked 2026-10-03: Beginner 50:00 -&gt; 49:30, at the US Army AFT 12 km bike pass scaled to 20 km (49:32 — it was 28 s easier than the Army minimum); a TT bike, flat, still air (tpf-app plan 61 Part C §4)</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -4826,7 +4838,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>103:30</t>
+          <t>102:30</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -6015,7 +6027,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no openly licensed study exists to check it against (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 (tpf-app plan 61 Part A §4.5): Experienced 18 ≈ Kliszczewicz 2014's mixed group (17.8 rounds, CC BY); Advanced 23 ≈ Butcher 2015's Open / Regional athletes (23.3, CC BY-NC — cross-check only). Elite 25 kept (whether it should be 28 is an open owner question in the app's record)</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -6076,7 +6088,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no openly licensed study exists to check it against (a gap)</t>
+          <t>TPF's own (expert-set), kept and checked 2026-10-03 (tpf-app plan 61 Part A §4.4): women's / men's 0.83-0.91 (mean 0.88), inside the CrossFit evidence — Toledo 2021 0.94 and Mangine 2018 (Fight Gone Bad) 0.87, both CC BY; Kliszczewicz 2014's entry floor 0.71, CC BY; Forte 2022 0.95, CC BY-NC-ND, cross-check only. The levels agree: Forte's women averaged 15.7 rounds (Experienced 16); Kliszczewicz's women's floor is 10 (Beginner)</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -6244,12 +6256,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1:35:00</t>
+          <t>1:57:30</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1:30:30</t>
+          <t>1:37:30</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -6279,7 +6291,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Elite: Rappelt et al. 2026 (Front Physiol, CC BY), season-7 ELITE-division median (57:17) x 1.187; lower tiers TPF's own (provisional — need the owner's numbers). Numbers unchanged 2026-10-02</t>
+          <t>Elite: Rappelt et al. 2026 (Front Physiol, CC BY), season-7 ELITE-division median (57:17) x 1.187. Advanced: the median PRO racer of season 7 at Open weights (Rappelt Figure 2, x 0.93 for the lighter Open stations — TPF judgement) 1:14:28, kept 1:14:00. Intermediate: TPF's own, between the anchors. Experienced: Brandt et al. 2025 (Front Physiol, CC BY), recreational Open median 86.5 min, kept 1:26:00. Novice / Beginner: 3.9 x TPF's own 5 km Novice / Beginner (25:00 / 30:05; HYROX time scales with running, Rappelt and Brandt), rounded to 30 s: 1:37:30 / 1:57:30 (were 1:30:30 / 1:35:00). Mirrors tpf-app plan 61 Part A §3.4 (2026-10-03)</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -6319,17 +6331,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1:44:30</t>
+          <t>2:09:30</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1:39:30</t>
+          <t>1:47:30</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1:35:00</t>
+          <t>1:34:30</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -6354,7 +6366,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Elite: Rappelt et al. 2026 (Front Physiol, CC BY), season-7 ELITE-division median (1:03:22) x 1.187 = 1:15:13, shown 1:15:00; lower tiers TPF's own (provisional), keeping the old spacing to elite. Rebuilt 2026-10-02</t>
+          <t>Women = men x 1.10 (Rappelt ELITE 1.106, PRO top-100 1.110), rounded to 30 s: Beginner 2:09:30, Novice 1:47:30, Experienced 1:34:30 (were 1:44:30 / 1:39:30 / 1:35:00); Intermediate 1:28:00 and Advanced 1:21:30 kept; Elite = Rappelt et al. 2026 (Front Physiol, CC BY) season-7 ELITE-division median (1:03:22) x 1.187 = 1:15:13, shown 1:15:00. Mirrors tpf-app plan 61 Part A §3.4 (2026-10-03)</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">

</xml_diff>

<commit_message>
Standards research in lockstep with the app (plan 61, 2026-10-03) (#6)
- Operator (scripts/apply-standards-research-2026-10-03.py, expect-then-set
  guards): Pararescue on the 2023 IFT (run 10:20, swim 12:30, push-ups 40,
  sit-ups 50, pull-ups "(2 min)"), broad jump (general 1.70/1.95/2.20/2.40,
  special forces 1.93/2.16/2.39/2.65), police plank 1:30/2:30/3:30/4:30, USMC
  plank Pass 1:10; the app's cites copied into a new cite column.
- Lift: HYROX Open lower tiers (men and women), Cindy's note, the site's own
  broad jump men's Elite 2.85 -> 2.75, and three base cells the app moved
  (women's OHP Beginner 25 kg, women's 20 / 40 km TT Beginner).
- New check:app-lift (WODs, base table, pathway overrides vs the app);
  check:app-ors also compares cites. Both: 0 differences.

Co-authored-by: TGW7 <274256682+TGW7@users.noreply.github.com>
Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
+++ b/config/standards/TPF_HRS_Standards_v0_2026-06-21.xlsx
@@ -451,7 +451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,6 +551,18 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Cream-filled cell = value to be populated (TODO). Red text = legal/commercial caution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Change 2026-10-03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Mirrors the TPF app's plan 61 (tpf-app docs/build/61_MISSING_STANDARDS_RESEARCH_2026-10-03.md section 8). HYROX race: men Beginner 1:57:30 and Novice 1:37:30 (3.9 x TPF's 5 km), women Beginner 2:09:30, Novice 1:47:30, Experienced 1:34:30 (men x 1.10); every tier now has a permitted basis. Cindy kept, now checked. TPF Benchmark's own broad jump: men's Elite 285 -&gt; 275 cm, relabelled TPF's own, now checked. The HABS base table follows the app: women's overhead press Beginner 20 -&gt; 25 kg, women's 20 km TT Beginner 50:00 -&gt; 49:30 (40 km derived: 1:42:30). Script: scripts/apply-standards-research-2026-10-03.py.</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1160,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>TPF's own ladder. No openly licensed population norm exists; checked only against published ratios (women's overhead press ≈ 0.5-0.6 of men's absolute — Nuzzo 2023 review) and the CrossFit sample of Meier, Rabel, Schmidt 2021 (Sports 9:80, CC BY)</t>
+          <t>TPF's own ladder. No openly licensed population norm exists. Checked 2026-10-03 (tpf-app plan 61 Part C §2.2) against TPF's own bench / squat / deadlift ladders x the overhead-press ratios of the CrossFit samples of Meier, Rabel, Schmidt 2021 (Sports 9:80) and Dexheimer 2019 (both CC BY): the men's ladder reproduced to within 2.5 kg; the women's Beginner 20 -&gt; 25 kg (the empty bar sat below every anchor, 23-30 kg). Women's ≈ 0.5-0.6 of men's absolute (Nuzzo 2023 review)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1168,7 +1180,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Owner-set; ratio checks only (2026-10-02)</t>
+          <t>Owner-set; ratio checks (2026-10-03)</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1448,7 +1460,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set). No openly licensed population table has been checked yet (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 (tpf-app plan 61 Part B §3.3) against Norwegian conscripts 2020 (Aandstad et al. 2023, Scand J Med Sci Sports, CC BY 4.0), US Army Ranger course candidates (Physiol Rep 2026, CC BY), Serbian police students (through a CC BY review, Healthcare 2023), AFSPECWAR candidates (Feeney et al. 2023, facts) and China's National Student Physical Health Standard (2014 revision, a Ministry of Education standard). Men's Elite 285 -&gt; 275 cm (2.85 m sat above every anchor); the women's ladder kept, about 0.80 x the men's at every tier</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1468,7 +1480,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Expert-set (TPF)</t>
+          <t>Expert-set (TPF); checked against permitted anchors (2026-10-03)</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -2103,7 +2115,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>TPF's own triathlete-pathway anchor (round 13: elite 27:00 M ≈ 44 km/h). No permitted anchor yet (a gap)</t>
+          <t>TPF's own triathlete-pathway anchor (round 13: elite 27:00 M ≈ 44 km/h), checked 2026-10-03 (tpf-app plan 61 Part C §4): Beginner at the US Army AFT 12 km stationary-bike pass time (2025 tables, a US government work) scaled to 20 km (Riegel exp 1.05) — men 45:10, women 49:32, so the women's Beginner moved 50:00 -&gt; 49:30; Elite graded against the UCI Hour Records (facts) — men's Elite 74 % of world best; sex gap 1.11. Assumes a time-trial bike (or clip-on aero bars), a flat course and still air</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2123,7 +2135,7 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Owner-set (TPF)</t>
+          <t>Owner-set (TPF); checked against permitted anchors (2026-10-03)</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -3190,7 +3202,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>TPF's own; no openly licensed norm — ratio checks only (2026-10-02)</t>
+          <t>TPF's own; no openly licensed norm — checked 2026-10-03 against the CrossFit overhead-press ratios (Meier 2021, Dexheimer 2019, CC BY): reproduced to within 2.5 kg, kept (tpf-app plan 61 Part C §2.2)</t>
         </is>
       </c>
     </row>
@@ -3214,7 +3226,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F20" t="n">
         <v>30</v>
@@ -3236,7 +3248,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>TPF's own; no openly licensed norm — ratio checks only (2026-10-02)</t>
+          <t>TPF's own; no openly licensed norm — checked 2026-10-03 against the CrossFit overhead-press ratios (Meier 2021, Dexheimer 2019, CC BY): Beginner 20 -&gt; 25 kg, the empty bar sat below every anchor (tpf-app plan 61 Part C §2.2). The HYROX, triathlete and bodybuilder pathways keep their own 20 kg (an owner question in the app's record)</t>
         </is>
       </c>
     </row>
@@ -3646,16 +3658,16 @@
         <v>270</v>
       </c>
       <c r="K29" t="n">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no permitted table checked yet (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 against permitted anchors (Norwegian conscripts, Aandstad 2023, CC BY; US Army Ranger candidates, 2026, CC BY; China's student standard, 2014) — tpf-app plan 61 Part B §3.3</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>novice/intermediate/advanced interpolated from pass/good/excellent/elite (2026-08-07)</t>
+          <t>novice/intermediate/advanced interpolated from pass/good/excellent/elite (2026-08-07); Elite 285 -&gt; 275 cm 2026-10-03 (tpf-app plan 61 Part B §3.3: 2.85 m sat above every anchor; the women's 220 keeps a 0.80 ratio)</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3713,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no permitted table checked yet (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 against permitted anchors (Norwegian conscripts, Aandstad 2023, CC BY; US Army Ranger candidates, 2026, CC BY; China's student standard, 2014) — tpf-app plan 61 Part B §3.3</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4666,7 +4678,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>TPF's own (round 13); no permitted anchor yet (a gap)</t>
+          <t>TPF's own (round 13); checked 2026-10-03: Beginner at the US Army AFT 12 km bike pass scaled to 20 km (45:10), Elite graded against the UCI Hour Records; a TT bike, flat, still air (tpf-app plan 61 Part C §4)</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -4696,7 +4708,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>50:00</t>
+          <t>49:30</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4731,7 +4743,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>TPF's own (round 13); no permitted anchor yet (a gap)</t>
+          <t>TPF's own (round 13); checked 2026-10-03: Beginner 50:00 -&gt; 49:30, at the US Army AFT 12 km bike pass scaled to 20 km (49:32 — it was 28 s easier than the Army minimum); a TT bike, flat, still air (tpf-app plan 61 Part C §4)</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -4826,7 +4838,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>103:30</t>
+          <t>102:30</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -6015,7 +6027,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no openly licensed study exists to check it against (a gap)</t>
+          <t>TPF's own (expert-set), checked 2026-10-03 (tpf-app plan 61 Part A §4.5): Experienced 18 ≈ Kliszczewicz 2014's mixed group (17.8 rounds, CC BY); Advanced 23 ≈ Butcher 2015's Open / Regional athletes (23.3, CC BY-NC — cross-check only). Elite 25 kept (whether it should be 28 is an open owner question in the app's record)</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -6076,7 +6088,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>TPF's own (expert-set); no openly licensed study exists to check it against (a gap)</t>
+          <t>TPF's own (expert-set), kept and checked 2026-10-03 (tpf-app plan 61 Part A §4.4): women's / men's 0.83-0.91 (mean 0.88), inside the CrossFit evidence — Toledo 2021 0.94 and Mangine 2018 (Fight Gone Bad) 0.87, both CC BY; Kliszczewicz 2014's entry floor 0.71, CC BY; Forte 2022 0.95, CC BY-NC-ND, cross-check only. The levels agree: Forte's women averaged 15.7 rounds (Experienced 16); Kliszczewicz's women's floor is 10 (Beginner)</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -6244,12 +6256,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1:35:00</t>
+          <t>1:57:30</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>1:30:30</t>
+          <t>1:37:30</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -6279,7 +6291,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Elite: Rappelt et al. 2026 (Front Physiol, CC BY), season-7 ELITE-division median (57:17) x 1.187; lower tiers TPF's own (provisional — need the owner's numbers). Numbers unchanged 2026-10-02</t>
+          <t>Elite: Rappelt et al. 2026 (Front Physiol, CC BY), season-7 ELITE-division median (57:17) x 1.187. Advanced: the median PRO racer of season 7 at Open weights (Rappelt Figure 2, x 0.93 for the lighter Open stations — TPF judgement) 1:14:28, kept 1:14:00. Intermediate: TPF's own, between the anchors. Experienced: Brandt et al. 2025 (Front Physiol, CC BY), recreational Open median 86.5 min, kept 1:26:00. Novice / Beginner: 3.9 x TPF's own 5 km Novice / Beginner (25:00 / 30:05; HYROX time scales with running, Rappelt and Brandt), rounded to 30 s: 1:37:30 / 1:57:30 (were 1:30:30 / 1:35:00). Mirrors tpf-app plan 61 Part A §3.4 (2026-10-03)</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -6319,17 +6331,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1:44:30</t>
+          <t>2:09:30</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>1:39:30</t>
+          <t>1:47:30</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>1:35:00</t>
+          <t>1:34:30</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -6354,7 +6366,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Elite: Rappelt et al. 2026 (Front Physiol, CC BY), season-7 ELITE-division median (1:03:22) x 1.187 = 1:15:13, shown 1:15:00; lower tiers TPF's own (provisional), keeping the old spacing to elite. Rebuilt 2026-10-02</t>
+          <t>Women = men x 1.10 (Rappelt ELITE 1.106, PRO top-100 1.110), rounded to 30 s: Beginner 2:09:30, Novice 1:47:30, Experienced 1:34:30 (were 1:44:30 / 1:39:30 / 1:35:00); Intermediate 1:28:00 and Advanced 1:21:30 kept; Elite = Rappelt et al. 2026 (Front Physiol, CC BY) season-7 ELITE-division median (1:03:22) x 1.187 = 1:15:13, shown 1:15:00. Mirrors tpf-app plan 61 Part A §3.4 (2026-10-03)</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">

</xml_diff>